<commit_message>
[ADD] Hyperparams template, beginning
</commit_message>
<xml_diff>
--- a/results/metrics_modelling2_highlight.xlsx
+++ b/results/metrics_modelling2_highlight.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vulf/Git/Hub/Drop_wall_impact/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\dropwall_impact\Drop_wall_impact\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828C9776-69BA-2742-9620-BA516FD283EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFF3A57-33CE-4F50-915F-8416125BAE35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Net Impact" sheetId="2" r:id="rId1"/>
@@ -233,20 +233,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -546,18 +545,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{010EC710-5209-3843-AF23-07065BB07E1C}">
-  <sheetPr codeName="Sheet2" filterMode="1"/>
-  <dimension ref="A1:H98"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:H97"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -582,7 +581,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -608,7 +607,7 @@
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -634,7 +633,7 @@
         <v>0.93181818181818177</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>43</v>
       </c>
@@ -660,7 +659,7 @@
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>44</v>
       </c>
@@ -686,7 +685,7 @@
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>44</v>
       </c>
@@ -712,33 +711,33 @@
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="5" t="s">
+    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>0.94666666666666666</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>0.9</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>0.9</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>0.9</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <v>0.93181818181818177</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>44</v>
       </c>
@@ -764,7 +763,7 @@
         <v>0.84722222222222221</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>44</v>
       </c>
@@ -790,7 +789,7 @@
         <v>0.82060185185185186</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>44</v>
       </c>
@@ -816,7 +815,7 @@
         <v>0.82870370370370361</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -842,7 +841,7 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -868,7 +867,7 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -894,7 +893,7 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>44</v>
       </c>
@@ -920,7 +919,7 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
@@ -946,7 +945,7 @@
         <v>0.81018518518518512</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -972,59 +971,59 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="5" t="s">
+    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>0.93333333333333335</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="4">
         <v>0.87804878048780477</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="4">
         <v>0.8571428571428571</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="4">
         <v>0.9</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="5" t="s">
+    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>0.93333333333333335</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <v>0.87804878048780477</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="4">
         <v>0.8571428571428571</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="4">
         <v>0.9</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>43</v>
       </c>
@@ -1050,7 +1049,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>44</v>
       </c>
@@ -1076,7 +1075,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -1102,7 +1101,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>44</v>
       </c>
@@ -1128,7 +1127,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -1154,7 +1153,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1180,7 +1179,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -1206,7 +1205,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1232,7 +1231,7 @@
         <v>0.90681818181818186</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -1258,33 +1257,33 @@
         <v>0.90681818181818186</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="3" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28">
         <v>0.84</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28">
         <v>0.86956521739130432</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28">
         <v>0.90909090909090906</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28">
         <v>0.84259259259259256</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -1310,7 +1309,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -1336,7 +1335,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -1362,7 +1361,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -1388,7 +1387,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1414,7 +1413,7 @@
         <v>0.80787037037037035</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -1440,7 +1439,7 @@
         <v>0.80787037037037035</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -1466,7 +1465,7 @@
         <v>0.76504629629629628</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -1492,7 +1491,7 @@
         <v>0.82407407407407418</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1518,7 +1517,7 @@
         <v>0.82407407407407418</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -1544,7 +1543,7 @@
         <v>0.78935185185185186</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>43</v>
       </c>
@@ -1570,7 +1569,7 @@
         <v>0.91363636363636358</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1596,7 +1595,7 @@
         <v>0.74652777777777768</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -1622,7 +1621,7 @@
         <v>0.74652777777777768</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -1648,7 +1647,7 @@
         <v>0.75462962962962954</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>43</v>
       </c>
@@ -1674,7 +1673,7 @@
         <v>0.75462962962962954</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -1700,7 +1699,7 @@
         <v>0.80555555555555558</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -1726,7 +1725,7 @@
         <v>0.73611111111111116</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>43</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>0.73611111111111116</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -1778,7 +1777,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1804,7 +1803,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>43</v>
       </c>
@@ -1830,7 +1829,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -1856,7 +1855,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>43</v>
       </c>
@@ -1882,7 +1881,7 @@
         <v>0.74421296296296302</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>44</v>
       </c>
@@ -1908,7 +1907,7 @@
         <v>0.88181818181818183</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -1934,7 +1933,7 @@
         <v>0.78703703703703709</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>43</v>
       </c>
@@ -1960,7 +1959,7 @@
         <v>0.78703703703703709</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>43</v>
       </c>
@@ -1986,7 +1985,7 @@
         <v>0.79513888888888895</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -2012,7 +2011,7 @@
         <v>0.72569444444444453</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>43</v>
       </c>
@@ -2038,7 +2037,7 @@
         <v>0.7685185185185186</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>44</v>
       </c>
@@ -2064,7 +2063,7 @@
         <v>0.7685185185185186</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -2090,7 +2089,7 @@
         <v>0.88863636363636367</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>43</v>
       </c>
@@ -2116,7 +2115,7 @@
         <v>0.74189814814814814</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>44</v>
       </c>
@@ -2142,7 +2141,7 @@
         <v>0.74189814814814814</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -2168,33 +2167,33 @@
         <v>0.91136363636363638</v>
       </c>
     </row>
-    <row r="63" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C63" s="5" t="s">
+    <row r="63" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C63" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D63" s="5">
+      <c r="D63" s="4">
         <v>0.89333333333333331</v>
       </c>
-      <c r="E63" s="5">
+      <c r="E63" s="4">
         <v>0.82608695652173925</v>
       </c>
-      <c r="F63" s="5">
+      <c r="F63" s="4">
         <v>0.73076923076923073</v>
       </c>
-      <c r="G63" s="5">
+      <c r="G63" s="4">
         <v>0.95</v>
       </c>
-      <c r="H63" s="5">
+      <c r="H63" s="4">
         <v>0.91136363636363638</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -2220,7 +2219,7 @@
         <v>0.8727272727272728</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -2246,59 +2245,59 @@
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C66" s="5" t="s">
+    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C66" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D66" s="5">
+      <c r="D66" s="4">
         <v>0.89333333333333331</v>
       </c>
-      <c r="E66" s="5">
+      <c r="E66" s="4">
         <v>0.80000000000000016</v>
       </c>
-      <c r="F66" s="5">
+      <c r="F66" s="4">
         <v>0.8</v>
       </c>
-      <c r="G66" s="5">
+      <c r="G66" s="4">
         <v>0.8</v>
       </c>
-      <c r="H66" s="5">
+      <c r="H66" s="4">
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="67" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C67" s="5" t="s">
+    <row r="67" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C67" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D67" s="5">
+      <c r="D67" s="4">
         <v>0.89333333333333331</v>
       </c>
-      <c r="E67" s="5">
+      <c r="E67" s="4">
         <v>0.80000000000000016</v>
       </c>
-      <c r="F67" s="5">
+      <c r="F67" s="4">
         <v>0.8</v>
       </c>
-      <c r="G67" s="5">
+      <c r="G67" s="4">
         <v>0.8</v>
       </c>
-      <c r="H67" s="5">
+      <c r="H67" s="4">
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>43</v>
       </c>
@@ -2324,7 +2323,7 @@
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>44</v>
       </c>
@@ -2350,33 +2349,33 @@
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C70" s="5" t="s">
+    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C70" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D70" s="5">
+      <c r="D70" s="4">
         <v>0.88</v>
       </c>
-      <c r="E70" s="5">
+      <c r="E70" s="4">
         <v>0.79999999999999993</v>
       </c>
-      <c r="F70" s="5">
+      <c r="F70" s="4">
         <v>0.72</v>
       </c>
-      <c r="G70" s="5">
+      <c r="G70" s="4">
         <v>0.9</v>
       </c>
-      <c r="H70" s="5">
+      <c r="H70" s="4">
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -2402,7 +2401,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>44</v>
       </c>
@@ -2428,7 +2427,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>44</v>
       </c>
@@ -2454,7 +2453,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>43</v>
       </c>
@@ -2480,7 +2479,7 @@
         <v>0.84772727272727277</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -2506,7 +2505,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -2532,7 +2531,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>43</v>
       </c>
@@ -2558,7 +2557,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>44</v>
       </c>
@@ -2584,7 +2583,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -2610,7 +2609,7 @@
         <v>0.8545454545454545</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>43</v>
       </c>
@@ -2636,7 +2635,7 @@
         <v>0.8545454545454545</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -2662,7 +2661,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>43</v>
       </c>
@@ -2688,7 +2687,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>44</v>
       </c>
@@ -2714,7 +2713,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>44</v>
       </c>
@@ -2740,7 +2739,7 @@
         <v>0.83863636363636351</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -2766,7 +2765,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>43</v>
       </c>
@@ -2792,7 +2791,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>43</v>
       </c>
@@ -2818,7 +2817,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>44</v>
       </c>
@@ -2844,7 +2843,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -2870,7 +2869,7 @@
         <v>0.85227272727272718</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>44</v>
       </c>
@@ -2896,7 +2895,7 @@
         <v>0.85227272727272718</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>44</v>
       </c>
@@ -2922,7 +2921,7 @@
         <v>0.85909090909090902</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>43</v>
       </c>
@@ -2948,7 +2947,7 @@
         <v>0.80681818181818177</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>43</v>
       </c>
@@ -2974,7 +2973,7 @@
         <v>0.84318181818181825</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -3000,7 +2999,7 @@
         <v>0.81363636363636349</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -3026,7 +3025,7 @@
         <v>0.83409090909090911</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>44</v>
       </c>
@@ -3052,7 +3051,7 @@
         <v>0.79772727272727262</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>44</v>
       </c>
@@ -3078,21 +3077,8 @@
         <v>0.78863636363636358</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A1:H98" xr:uid="{010EC710-5209-3843-AF23-07065BB07E1C}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="df_modelling_dimensionless"/>
-        <filter val="df_modelling_no_multicollinearity"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="net_impact"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H98" xr:uid="{010EC710-5209-3843-AF23-07065BB07E1C}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3102,15 +3088,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1" filterMode="1"/>
   <dimension ref="A1:H98"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3136,7 +3122,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3162,7 +3148,7 @@
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3188,85 +3174,85 @@
         <v>0.93181818181818177</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="5" t="s">
+    <row r="4" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>0.8666666666666667</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>0.9</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>0.86538461538461542</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>0.9375</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="5" t="s">
+    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>0.8666666666666667</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>0.9</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>0.86538461538461542</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>0.9375</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="5" t="s">
+    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>0.8666666666666667</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>0.9</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>0.86538461538461542</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>0.9375</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <v>0.83912037037037035</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -3292,7 +3278,7 @@
         <v>0.93181818181818177</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>44</v>
       </c>
@@ -3318,7 +3304,7 @@
         <v>0.84722222222222221</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>44</v>
       </c>
@@ -3344,33 +3330,33 @@
         <v>0.82060185185185186</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="5" t="s">
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>0.85333333333333339</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>0.88888888888888895</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <v>0.86274509803921573</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>0.91666666666666663</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <v>0.82870370370370361</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -3396,7 +3382,7 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -3422,33 +3408,33 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="5" t="s">
+    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>0.85333333333333339</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <v>0.88659793814432986</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <v>0.87755102040816324</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>0.89583333333333337</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>44</v>
       </c>
@@ -3474,33 +3460,33 @@
         <v>0.83680555555555558</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="5" t="s">
+    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>0.84</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <v>0.87999999999999989</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <v>0.84615384615384615</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="4">
         <v>0.91666666666666663</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <v>0.81018518518518512</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -3526,7 +3512,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -3552,7 +3538,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -3578,7 +3564,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -3604,7 +3590,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -3630,7 +3616,7 @@
         <v>0.92272727272727262</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -3656,33 +3642,33 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="5" t="s">
+    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
         <v>0.84</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="4">
         <v>0.87755102040816324</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="4">
         <v>0.86</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="4">
         <v>0.89583333333333337</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="4">
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -3708,7 +3694,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -3734,7 +3720,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -3760,7 +3746,7 @@
         <v>0.81828703703703709</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -3786,7 +3772,7 @@
         <v>0.90681818181818186</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -3812,33 +3798,33 @@
         <v>0.90681818181818186</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="3" t="s">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28">
         <v>0.84</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28">
         <v>0.86956521739130432</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28">
         <v>0.90909090909090906</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28">
         <v>0.84259259259259256</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -3864,7 +3850,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -3890,7 +3876,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -3916,7 +3902,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -3942,7 +3928,7 @@
         <v>0.7997685185185186</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -3968,7 +3954,7 @@
         <v>0.80787037037037035</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -3994,7 +3980,7 @@
         <v>0.80787037037037035</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -4020,7 +4006,7 @@
         <v>0.76504629629629628</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -4046,7 +4032,7 @@
         <v>0.82407407407407418</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -4072,7 +4058,7 @@
         <v>0.82407407407407418</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -4098,7 +4084,7 @@
         <v>0.78935185185185186</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -4124,7 +4110,7 @@
         <v>0.91363636363636358</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -4150,7 +4136,7 @@
         <v>0.74652777777777768</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -4176,7 +4162,7 @@
         <v>0.74652777777777768</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -4202,7 +4188,7 @@
         <v>0.75462962962962954</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>43</v>
       </c>
@@ -4228,7 +4214,7 @@
         <v>0.75462962962962954</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -4254,7 +4240,7 @@
         <v>0.80555555555555558</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -4280,7 +4266,7 @@
         <v>0.73611111111111116</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>43</v>
       </c>
@@ -4306,7 +4292,7 @@
         <v>0.73611111111111116</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -4332,7 +4318,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -4358,7 +4344,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>43</v>
       </c>
@@ -4384,7 +4370,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>43</v>
       </c>
@@ -4410,7 +4396,7 @@
         <v>0.77893518518518512</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>43</v>
       </c>
@@ -4436,7 +4422,7 @@
         <v>0.74421296296296302</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>44</v>
       </c>
@@ -4462,7 +4448,7 @@
         <v>0.88181818181818183</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -4488,7 +4474,7 @@
         <v>0.78703703703703709</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>43</v>
       </c>
@@ -4514,7 +4500,7 @@
         <v>0.78703703703703709</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>43</v>
       </c>
@@ -4540,7 +4526,7 @@
         <v>0.79513888888888895</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -4566,7 +4552,7 @@
         <v>0.72569444444444453</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>43</v>
       </c>
@@ -4592,7 +4578,7 @@
         <v>0.7685185185185186</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>44</v>
       </c>
@@ -4618,7 +4604,7 @@
         <v>0.7685185185185186</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -4644,7 +4630,7 @@
         <v>0.88863636363636367</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>43</v>
       </c>
@@ -4670,7 +4656,7 @@
         <v>0.74189814814814814</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>44</v>
       </c>
@@ -4696,7 +4682,7 @@
         <v>0.74189814814814814</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -4722,7 +4708,7 @@
         <v>0.91136363636363638</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>43</v>
       </c>
@@ -4748,7 +4734,7 @@
         <v>0.91136363636363638</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -4774,7 +4760,7 @@
         <v>0.8727272727272728</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -4800,7 +4786,7 @@
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>43</v>
       </c>
@@ -4826,7 +4812,7 @@
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>44</v>
       </c>
@@ -4852,7 +4838,7 @@
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>43</v>
       </c>
@@ -4878,7 +4864,7 @@
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>44</v>
       </c>
@@ -4904,7 +4890,7 @@
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>44</v>
       </c>
@@ -4930,7 +4916,7 @@
         <v>0.88636363636363635</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -4956,7 +4942,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>44</v>
       </c>
@@ -4982,7 +4968,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>44</v>
       </c>
@@ -5008,7 +4994,7 @@
         <v>0.87045454545454548</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>43</v>
       </c>
@@ -5034,7 +5020,7 @@
         <v>0.84772727272727277</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -5060,7 +5046,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -5086,7 +5072,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>43</v>
       </c>
@@ -5112,7 +5098,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>44</v>
       </c>
@@ -5138,7 +5124,7 @@
         <v>0.8772727272727272</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -5164,7 +5150,7 @@
         <v>0.8545454545454545</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>43</v>
       </c>
@@ -5190,7 +5176,7 @@
         <v>0.8545454545454545</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -5216,7 +5202,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>43</v>
       </c>
@@ -5242,7 +5228,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>44</v>
       </c>
@@ -5268,7 +5254,7 @@
         <v>0.83181818181818179</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>44</v>
       </c>
@@ -5294,7 +5280,7 @@
         <v>0.83863636363636351</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -5320,7 +5306,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>43</v>
       </c>
@@ -5346,7 +5332,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>43</v>
       </c>
@@ -5372,7 +5358,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>44</v>
       </c>
@@ -5398,7 +5384,7 @@
         <v>0.86818181818181817</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -5424,7 +5410,7 @@
         <v>0.85227272727272718</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>44</v>
       </c>
@@ -5450,7 +5436,7 @@
         <v>0.85227272727272718</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>44</v>
       </c>
@@ -5476,7 +5462,7 @@
         <v>0.85909090909090902</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>43</v>
       </c>
@@ -5502,7 +5488,7 @@
         <v>0.80681818181818177</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>43</v>
       </c>
@@ -5528,7 +5514,7 @@
         <v>0.84318181818181825</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -5554,7 +5540,7 @@
         <v>0.81363636363636349</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -5580,7 +5566,7 @@
         <v>0.83409090909090911</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>44</v>
       </c>
@@ -5606,7 +5592,7 @@
         <v>0.79772727272727262</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>44</v>
       </c>
@@ -5632,7 +5618,7 @@
         <v>0.78863636363636358</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <autoFilter ref="A1:H98" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">

</xml_diff>